<commit_message>
add fig 1 and fig 2
</commit_message>
<xml_diff>
--- a/data/Master+Namen.xlsx
+++ b/data/Master+Namen.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utexas-my.sharepoint.com/personal/txe_mail_utexas_edu/Documents/RStudio/dollinger/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utexas-my.sharepoint.com/personal/lh9896_eid_utexas_edu/Documents/RStudio/dollinger/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{1746B2BE-BE8A-6B48-8CC8-C16ABDA29276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6B0D8EF-752C-7249-89E1-4D5B1C7188E4}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{1746B2BE-BE8A-6B48-8CC8-C16ABDA29276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{03AF0456-86F9-0D41-81FB-785715D79E28}"/>
   <bookViews>
-    <workbookView xWindow="19340" yWindow="9080" windowWidth="38360" windowHeight="18420" xr2:uid="{6A40146A-9B1A-1645-A6CD-02795C3C9332}"/>
+    <workbookView xWindow="40600" yWindow="-9360" windowWidth="19340" windowHeight="37460" xr2:uid="{6A40146A-9B1A-1645-A6CD-02795C3C9332}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,11 +27,34 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1023,12 +1046,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82931FF0-30E7-0E43-816A-AE731A8B3A34}">
-  <dimension ref="A1:AK18"/>
+  <dimension ref="A1:AK56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.1640625" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" customWidth="1"/>
+    <col min="3" max="3" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="36.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="37.1640625" bestFit="1" customWidth="1"/>
@@ -2247,7 +2271,2081 @@
         <v>172</v>
       </c>
     </row>
+    <row r="20" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A20" t="str" cm="1">
+        <f t="array" ref="A20:R56">TRANSPOSE(A1:AK18)</f>
+        <v>Kurzname</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Langfrage</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Werte</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <v>0</v>
+      </c>
+      <c r="M20">
+        <v>0</v>
+      </c>
+      <c r="N20">
+        <v>0</v>
+      </c>
+      <c r="O20">
+        <v>0</v>
+      </c>
+      <c r="P20">
+        <v>0</v>
+      </c>
+      <c r="Q20">
+        <v>0</v>
+      </c>
+      <c r="R20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A21" t="str">
+        <v>Cool</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Q1</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Strongly disagree</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Disagree</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Somewhat disagree</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Don't know</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Somewhat agree</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Agree</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Strongly agree</v>
+      </c>
+      <c r="J21">
+        <v>0</v>
+      </c>
+      <c r="K21">
+        <v>0</v>
+      </c>
+      <c r="L21">
+        <v>0</v>
+      </c>
+      <c r="M21">
+        <v>0</v>
+      </c>
+      <c r="N21">
+        <v>0</v>
+      </c>
+      <c r="O21">
+        <v>0</v>
+      </c>
+      <c r="P21">
+        <v>0</v>
+      </c>
+      <c r="Q21">
+        <v>0</v>
+      </c>
+      <c r="R21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A22" t="str">
+        <v>Multiling</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Q2</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Definitely not</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Probably not</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Neutral</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Probably yes</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Definitely yes</v>
+      </c>
+      <c r="H22" t="str">
+        <v>× Don't know</v>
+      </c>
+      <c r="I22">
+        <v>0</v>
+      </c>
+      <c r="J22">
+        <v>0</v>
+      </c>
+      <c r="K22">
+        <v>0</v>
+      </c>
+      <c r="L22">
+        <v>0</v>
+      </c>
+      <c r="M22">
+        <v>0</v>
+      </c>
+      <c r="N22">
+        <v>0</v>
+      </c>
+      <c r="O22">
+        <v>0</v>
+      </c>
+      <c r="P22">
+        <v>0</v>
+      </c>
+      <c r="Q22">
+        <v>0</v>
+      </c>
+      <c r="R22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A23" t="str">
+        <v>Umultiling</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Q58</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D23" t="str">
+        <v>No</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+      <c r="L23">
+        <v>0</v>
+      </c>
+      <c r="M23">
+        <v>0</v>
+      </c>
+      <c r="N23">
+        <v>0</v>
+      </c>
+      <c r="O23">
+        <v>0</v>
+      </c>
+      <c r="P23">
+        <v>0</v>
+      </c>
+      <c r="Q23">
+        <v>0</v>
+      </c>
+      <c r="R23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A24" t="str">
+        <v>ComfNonEng</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Q13</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Extremely uncomfortable</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Moderately uncomfortable</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Neither comfortable nor uncomfortable</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Moderately comfortable</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Extremely comfortable</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Does not apply to me (I don't live in Canada)</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+      <c r="L24">
+        <v>0</v>
+      </c>
+      <c r="M24">
+        <v>0</v>
+      </c>
+      <c r="N24">
+        <v>0</v>
+      </c>
+      <c r="O24">
+        <v>0</v>
+      </c>
+      <c r="P24">
+        <v>0</v>
+      </c>
+      <c r="Q24">
+        <v>0</v>
+      </c>
+      <c r="R24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A25" t="str">
+        <v>Media</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Q14</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Extremely unimportant</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Unimportant</v>
+      </c>
+      <c r="E25" t="str">
+        <v>× Don't know</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Important</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Extremely important</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+      <c r="L25">
+        <v>0</v>
+      </c>
+      <c r="M25">
+        <v>0</v>
+      </c>
+      <c r="N25">
+        <v>0</v>
+      </c>
+      <c r="O25">
+        <v>0</v>
+      </c>
+      <c r="P25">
+        <v>0</v>
+      </c>
+      <c r="Q25">
+        <v>0</v>
+      </c>
+      <c r="R25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A26" t="str">
+        <v>Priv</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Q62</v>
+      </c>
+      <c r="C26" t="str">
+        <v>No</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E26" t="str">
+        <v>That depends (please also explain if you can)</v>
+      </c>
+      <c r="F26" t="str">
+        <v>× Don't know</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>0</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
+      <c r="L26">
+        <v>0</v>
+      </c>
+      <c r="M26">
+        <v>0</v>
+      </c>
+      <c r="N26">
+        <v>0</v>
+      </c>
+      <c r="O26">
+        <v>0</v>
+      </c>
+      <c r="P26">
+        <v>0</v>
+      </c>
+      <c r="Q26">
+        <v>0</v>
+      </c>
+      <c r="R26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A27" t="str">
+        <v>StHeard</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Q5</v>
+      </c>
+      <c r="C27" t="str">
+        <v>No</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Not sure</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+      <c r="L27">
+        <v>0</v>
+      </c>
+      <c r="M27">
+        <v>0</v>
+      </c>
+      <c r="N27">
+        <v>0</v>
+      </c>
+      <c r="O27">
+        <v>0</v>
+      </c>
+      <c r="P27">
+        <v>0</v>
+      </c>
+      <c r="Q27">
+        <v>0</v>
+      </c>
+      <c r="R27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A28" t="str">
+        <v>StDescr</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Q63</v>
+      </c>
+      <c r="C28" t="str">
+        <v>× No</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Yes, but I can't describe it well</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Yes, I do know. It is... (please describe briefly)</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28">
+        <v>0</v>
+      </c>
+      <c r="I28">
+        <v>0</v>
+      </c>
+      <c r="J28">
+        <v>0</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+      <c r="L28">
+        <v>0</v>
+      </c>
+      <c r="M28">
+        <v>0</v>
+      </c>
+      <c r="N28">
+        <v>0</v>
+      </c>
+      <c r="O28">
+        <v>0</v>
+      </c>
+      <c r="P28">
+        <v>0</v>
+      </c>
+      <c r="Q28">
+        <v>0</v>
+      </c>
+      <c r="R28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A29" t="str">
+        <v>Zed</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Q6</v>
+      </c>
+      <c r="C29" t="str">
+        <v>zed</v>
+      </c>
+      <c r="D29" t="str">
+        <v>zee</v>
+      </c>
+      <c r="E29" t="str">
+        <v>both</v>
+      </c>
+      <c r="F29" t="str">
+        <v>not sure</v>
+      </c>
+      <c r="G29">
+        <v>0</v>
+      </c>
+      <c r="H29">
+        <v>0</v>
+      </c>
+      <c r="I29">
+        <v>0</v>
+      </c>
+      <c r="J29">
+        <v>0</v>
+      </c>
+      <c r="K29">
+        <v>0</v>
+      </c>
+      <c r="L29">
+        <v>0</v>
+      </c>
+      <c r="M29">
+        <v>0</v>
+      </c>
+      <c r="N29">
+        <v>0</v>
+      </c>
+      <c r="O29">
+        <v>0</v>
+      </c>
+      <c r="P29">
+        <v>0</v>
+      </c>
+      <c r="Q29">
+        <v>0</v>
+      </c>
+      <c r="R29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A30" t="str">
+        <v>Spell</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Q18</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Very unimportant</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Unimportant</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Neither unimportant nor important</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Important</v>
+      </c>
+      <c r="G30" t="str">
+        <v>Very important</v>
+      </c>
+      <c r="H30" t="str">
+        <v>× Don't know</v>
+      </c>
+      <c r="I30">
+        <v>0</v>
+      </c>
+      <c r="J30">
+        <v>0</v>
+      </c>
+      <c r="K30">
+        <v>0</v>
+      </c>
+      <c r="L30">
+        <v>0</v>
+      </c>
+      <c r="M30">
+        <v>0</v>
+      </c>
+      <c r="N30">
+        <v>0</v>
+      </c>
+      <c r="O30">
+        <v>0</v>
+      </c>
+      <c r="P30">
+        <v>0</v>
+      </c>
+      <c r="Q30">
+        <v>0</v>
+      </c>
+      <c r="R30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A31" t="str">
+        <v>SpellUni</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Q19</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Very unimportant</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Unimportant</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Neither unimportant nor important</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Important</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Very important</v>
+      </c>
+      <c r="H31" t="str">
+        <v>× Don't know</v>
+      </c>
+      <c r="I31">
+        <v>0</v>
+      </c>
+      <c r="J31">
+        <v>0</v>
+      </c>
+      <c r="K31">
+        <v>0</v>
+      </c>
+      <c r="L31">
+        <v>0</v>
+      </c>
+      <c r="M31">
+        <v>0</v>
+      </c>
+      <c r="N31">
+        <v>0</v>
+      </c>
+      <c r="O31">
+        <v>0</v>
+      </c>
+      <c r="P31">
+        <v>0</v>
+      </c>
+      <c r="Q31">
+        <v>0</v>
+      </c>
+      <c r="R31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A32" t="str">
+        <v>Distinct</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Q4</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Definitely not</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Probably not</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Don't know</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Probably yes</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Definitely yes</v>
+      </c>
+      <c r="H32">
+        <v>0</v>
+      </c>
+      <c r="I32">
+        <v>0</v>
+      </c>
+      <c r="J32">
+        <v>0</v>
+      </c>
+      <c r="K32">
+        <v>0</v>
+      </c>
+      <c r="L32">
+        <v>0</v>
+      </c>
+      <c r="M32">
+        <v>0</v>
+      </c>
+      <c r="N32">
+        <v>0</v>
+      </c>
+      <c r="O32">
+        <v>0</v>
+      </c>
+      <c r="P32">
+        <v>0</v>
+      </c>
+      <c r="Q32">
+        <v>0</v>
+      </c>
+      <c r="R32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A33" t="str">
+        <v>SameEW</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Q8</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Definitely not</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Probably not</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Don't know</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Probably yes</v>
+      </c>
+      <c r="G33" t="str">
+        <v>Definitely yes</v>
+      </c>
+      <c r="H33">
+        <v>0</v>
+      </c>
+      <c r="I33">
+        <v>0</v>
+      </c>
+      <c r="J33">
+        <v>0</v>
+      </c>
+      <c r="K33">
+        <v>0</v>
+      </c>
+      <c r="L33">
+        <v>0</v>
+      </c>
+      <c r="M33">
+        <v>0</v>
+      </c>
+      <c r="N33">
+        <v>0</v>
+      </c>
+      <c r="O33">
+        <v>0</v>
+      </c>
+      <c r="P33">
+        <v>0</v>
+      </c>
+      <c r="Q33">
+        <v>0</v>
+      </c>
+      <c r="R33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A34" t="str">
+        <v>Celebs</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Q12</v>
+      </c>
+      <c r="C34" t="str">
+        <v>No</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Yes (please specify who):</v>
+      </c>
+      <c r="E34" t="str">
+        <v>× Don't know</v>
+      </c>
+      <c r="F34">
+        <v>0</v>
+      </c>
+      <c r="G34">
+        <v>0</v>
+      </c>
+      <c r="H34">
+        <v>0</v>
+      </c>
+      <c r="I34">
+        <v>0</v>
+      </c>
+      <c r="J34">
+        <v>0</v>
+      </c>
+      <c r="K34">
+        <v>0</v>
+      </c>
+      <c r="L34">
+        <v>0</v>
+      </c>
+      <c r="M34">
+        <v>0</v>
+      </c>
+      <c r="N34">
+        <v>0</v>
+      </c>
+      <c r="O34">
+        <v>0</v>
+      </c>
+      <c r="P34">
+        <v>0</v>
+      </c>
+      <c r="Q34">
+        <v>0</v>
+      </c>
+      <c r="R34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A35" t="str">
+        <v>Prestige</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Q10</v>
+      </c>
+      <c r="C35" t="str">
+        <v>American English</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Jamaican English</v>
+      </c>
+      <c r="E35" t="str">
+        <v>British English</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Canadian English</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Singaporean English</v>
+      </c>
+      <c r="H35" t="str">
+        <v>Irish English</v>
+      </c>
+      <c r="I35" t="str">
+        <v>Other (please name):</v>
+      </c>
+      <c r="J35" t="str">
+        <v>No particular variety</v>
+      </c>
+      <c r="K35">
+        <v>0</v>
+      </c>
+      <c r="L35">
+        <v>0</v>
+      </c>
+      <c r="M35">
+        <v>0</v>
+      </c>
+      <c r="N35">
+        <v>0</v>
+      </c>
+      <c r="O35">
+        <v>0</v>
+      </c>
+      <c r="P35">
+        <v>0</v>
+      </c>
+      <c r="Q35">
+        <v>0</v>
+      </c>
+      <c r="R35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A36" t="str">
+        <v>RecCdns</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Q15</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Always</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Often</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Sometimes</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Rarely</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Never</v>
+      </c>
+      <c r="H36" t="str">
+        <v>Don't know</v>
+      </c>
+      <c r="I36">
+        <v>0</v>
+      </c>
+      <c r="J36">
+        <v>0</v>
+      </c>
+      <c r="K36">
+        <v>0</v>
+      </c>
+      <c r="L36">
+        <v>0</v>
+      </c>
+      <c r="M36">
+        <v>0</v>
+      </c>
+      <c r="N36">
+        <v>0</v>
+      </c>
+      <c r="O36">
+        <v>0</v>
+      </c>
+      <c r="P36">
+        <v>0</v>
+      </c>
+      <c r="Q36">
+        <v>0</v>
+      </c>
+      <c r="R36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A37" t="str">
+        <v>Software</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Q17</v>
+      </c>
+      <c r="C37" t="str">
+        <v>No</v>
+      </c>
+      <c r="D37" t="str">
+        <v>× Don't know</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F37">
+        <v>0</v>
+      </c>
+      <c r="G37">
+        <v>0</v>
+      </c>
+      <c r="H37">
+        <v>0</v>
+      </c>
+      <c r="I37">
+        <v>0</v>
+      </c>
+      <c r="J37">
+        <v>0</v>
+      </c>
+      <c r="K37">
+        <v>0</v>
+      </c>
+      <c r="L37">
+        <v>0</v>
+      </c>
+      <c r="M37">
+        <v>0</v>
+      </c>
+      <c r="N37">
+        <v>0</v>
+      </c>
+      <c r="O37">
+        <v>0</v>
+      </c>
+      <c r="P37">
+        <v>0</v>
+      </c>
+      <c r="Q37">
+        <v>0</v>
+      </c>
+      <c r="R37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A38" t="str">
+        <v>Dictionary</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Q20</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Definitely not</v>
+      </c>
+      <c r="D38" t="str">
+        <v>No</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Neither yes or no</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Definitely yes</v>
+      </c>
+      <c r="H38" t="str">
+        <v>Don't know</v>
+      </c>
+      <c r="I38">
+        <v>0</v>
+      </c>
+      <c r="J38">
+        <v>0</v>
+      </c>
+      <c r="K38">
+        <v>0</v>
+      </c>
+      <c r="L38">
+        <v>0</v>
+      </c>
+      <c r="M38">
+        <v>0</v>
+      </c>
+      <c r="N38">
+        <v>0</v>
+      </c>
+      <c r="O38">
+        <v>0</v>
+      </c>
+      <c r="P38">
+        <v>0</v>
+      </c>
+      <c r="Q38">
+        <v>0</v>
+      </c>
+      <c r="R38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A39" t="str">
+        <v>RecogEh</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Q21</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Definitely not</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Probably not</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Might or might not</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Probably yes</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Definitely yes</v>
+      </c>
+      <c r="H39" t="str">
+        <v>× Don't know</v>
+      </c>
+      <c r="I39">
+        <v>0</v>
+      </c>
+      <c r="J39">
+        <v>0</v>
+      </c>
+      <c r="K39">
+        <v>0</v>
+      </c>
+      <c r="L39">
+        <v>0</v>
+      </c>
+      <c r="M39">
+        <v>0</v>
+      </c>
+      <c r="N39">
+        <v>0</v>
+      </c>
+      <c r="O39">
+        <v>0</v>
+      </c>
+      <c r="P39">
+        <v>0</v>
+      </c>
+      <c r="Q39">
+        <v>0</v>
+      </c>
+      <c r="R39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A40" t="str">
+        <v>Sorry</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Q23</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Definitely not</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Probably not</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Might or might not</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Probably yes</v>
+      </c>
+      <c r="G40" t="str">
+        <v>Definitely yes</v>
+      </c>
+      <c r="H40">
+        <v>0</v>
+      </c>
+      <c r="I40">
+        <v>0</v>
+      </c>
+      <c r="J40">
+        <v>0</v>
+      </c>
+      <c r="K40">
+        <v>0</v>
+      </c>
+      <c r="L40">
+        <v>0</v>
+      </c>
+      <c r="M40">
+        <v>0</v>
+      </c>
+      <c r="N40">
+        <v>0</v>
+      </c>
+      <c r="O40">
+        <v>0</v>
+      </c>
+      <c r="P40">
+        <v>0</v>
+      </c>
+      <c r="Q40">
+        <v>0</v>
+      </c>
+      <c r="R40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A41" t="str">
+        <v>EnglAble</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Q67a</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Strongly disagree</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Disagree</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Neither disagree or agree</v>
+      </c>
+      <c r="F41" t="str">
+        <v>Agree</v>
+      </c>
+      <c r="G41" t="str">
+        <v>Strongly agree</v>
+      </c>
+      <c r="H41" t="str">
+        <v>Don't know</v>
+      </c>
+      <c r="I41">
+        <v>0</v>
+      </c>
+      <c r="J41">
+        <v>0</v>
+      </c>
+      <c r="K41">
+        <v>0</v>
+      </c>
+      <c r="L41">
+        <v>0</v>
+      </c>
+      <c r="M41">
+        <v>0</v>
+      </c>
+      <c r="N41">
+        <v>0</v>
+      </c>
+      <c r="O41">
+        <v>0</v>
+      </c>
+      <c r="P41">
+        <v>0</v>
+      </c>
+      <c r="Q41">
+        <v>0</v>
+      </c>
+      <c r="R41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A42" t="str">
+        <v>FrAble</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Q67b</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Strongly disagree</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Disagree</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Neither disagree or agree</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Agree</v>
+      </c>
+      <c r="G42" t="str">
+        <v>Strongly agree</v>
+      </c>
+      <c r="H42" t="str">
+        <v>Don't know</v>
+      </c>
+      <c r="I42">
+        <v>0</v>
+      </c>
+      <c r="J42">
+        <v>0</v>
+      </c>
+      <c r="K42">
+        <v>0</v>
+      </c>
+      <c r="L42">
+        <v>0</v>
+      </c>
+      <c r="M42">
+        <v>0</v>
+      </c>
+      <c r="N42">
+        <v>0</v>
+      </c>
+      <c r="O42">
+        <v>0</v>
+      </c>
+      <c r="P42">
+        <v>0</v>
+      </c>
+      <c r="Q42">
+        <v>0</v>
+      </c>
+      <c r="R42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A43" t="str">
+        <v>IndAble</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Q67c</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Strongly disagree</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Disagree</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Neither disagree or agree</v>
+      </c>
+      <c r="F43" t="str">
+        <v>Agree</v>
+      </c>
+      <c r="G43" t="str">
+        <v>Strongly agree</v>
+      </c>
+      <c r="H43" t="str">
+        <v>Don't know</v>
+      </c>
+      <c r="I43">
+        <v>0</v>
+      </c>
+      <c r="J43">
+        <v>0</v>
+      </c>
+      <c r="K43">
+        <v>0</v>
+      </c>
+      <c r="L43">
+        <v>0</v>
+      </c>
+      <c r="M43">
+        <v>0</v>
+      </c>
+      <c r="N43">
+        <v>0</v>
+      </c>
+      <c r="O43">
+        <v>0</v>
+      </c>
+      <c r="P43">
+        <v>0</v>
+      </c>
+      <c r="Q43">
+        <v>0</v>
+      </c>
+      <c r="R43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A44" t="str">
+        <v>BeyondEF</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Q67d</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Strongly disagree</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Disagree</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Neither disagree or agree</v>
+      </c>
+      <c r="F44" t="str">
+        <v>Agree</v>
+      </c>
+      <c r="G44" t="str">
+        <v>Strongly agree</v>
+      </c>
+      <c r="H44" t="str">
+        <v>Don't know</v>
+      </c>
+      <c r="I44">
+        <v>0</v>
+      </c>
+      <c r="J44">
+        <v>0</v>
+      </c>
+      <c r="K44">
+        <v>0</v>
+      </c>
+      <c r="L44">
+        <v>0</v>
+      </c>
+      <c r="M44">
+        <v>0</v>
+      </c>
+      <c r="N44">
+        <v>0</v>
+      </c>
+      <c r="O44">
+        <v>0</v>
+      </c>
+      <c r="P44">
+        <v>0</v>
+      </c>
+      <c r="Q44">
+        <v>0</v>
+      </c>
+      <c r="R44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A45" t="str">
+        <v>CdnWay</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Q9</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Definitely not</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Probably not</v>
+      </c>
+      <c r="E45" t="str">
+        <v>× Don't know</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Probably yes</v>
+      </c>
+      <c r="G45" t="str">
+        <v>Definitely yes</v>
+      </c>
+      <c r="H45">
+        <v>0</v>
+      </c>
+      <c r="I45">
+        <v>0</v>
+      </c>
+      <c r="J45">
+        <v>0</v>
+      </c>
+      <c r="K45">
+        <v>0</v>
+      </c>
+      <c r="L45">
+        <v>0</v>
+      </c>
+      <c r="M45">
+        <v>0</v>
+      </c>
+      <c r="N45">
+        <v>0</v>
+      </c>
+      <c r="O45">
+        <v>0</v>
+      </c>
+      <c r="P45">
+        <v>0</v>
+      </c>
+      <c r="Q45">
+        <v>0</v>
+      </c>
+      <c r="R45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A46" t="str">
+        <v>Age</v>
+      </c>
+      <c r="B46">
+        <v>0</v>
+      </c>
+      <c r="C46" t="str">
+        <v>14 and under</v>
+      </c>
+      <c r="D46" t="str">
+        <v>15-19</v>
+      </c>
+      <c r="E46" t="str">
+        <v>20-24</v>
+      </c>
+      <c r="F46" t="str">
+        <v>25-29</v>
+      </c>
+      <c r="G46" t="str">
+        <v>30-34</v>
+      </c>
+      <c r="H46" t="str">
+        <v>35-39</v>
+      </c>
+      <c r="I46" t="str">
+        <v>40-44</v>
+      </c>
+      <c r="J46" t="str">
+        <v>45-49</v>
+      </c>
+      <c r="K46" t="str">
+        <v>50-54</v>
+      </c>
+      <c r="L46" t="str">
+        <v>55-59</v>
+      </c>
+      <c r="M46" t="str">
+        <v>60-64</v>
+      </c>
+      <c r="N46" t="str">
+        <v>65-69</v>
+      </c>
+      <c r="O46" t="str">
+        <v>70-74</v>
+      </c>
+      <c r="P46" t="str">
+        <v>75-79</v>
+      </c>
+      <c r="Q46" t="str">
+        <v>80-84</v>
+      </c>
+      <c r="R46" t="str">
+        <v>85-89</v>
+      </c>
+    </row>
+    <row r="47" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A47" t="str">
+        <v>LiveLand</v>
+      </c>
+      <c r="B47">
+        <v>0</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="D47" t="str">
+        <v>United States</v>
+      </c>
+      <c r="E47" t="str">
+        <v>United Kingdom</v>
+      </c>
+      <c r="F47" t="str">
+        <v>Australia</v>
+      </c>
+      <c r="G47">
+        <v>0</v>
+      </c>
+      <c r="H47" t="str">
+        <v>all others can be lumped as "Other"</v>
+      </c>
+      <c r="I47">
+        <v>0</v>
+      </c>
+      <c r="J47">
+        <v>0</v>
+      </c>
+      <c r="K47">
+        <v>0</v>
+      </c>
+      <c r="L47">
+        <v>0</v>
+      </c>
+      <c r="M47">
+        <v>0</v>
+      </c>
+      <c r="N47">
+        <v>0</v>
+      </c>
+      <c r="O47">
+        <v>0</v>
+      </c>
+      <c r="P47">
+        <v>0</v>
+      </c>
+      <c r="Q47">
+        <v>0</v>
+      </c>
+      <c r="R47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A48" t="str">
+        <v>LiveProv</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="str">
+        <v>10+3 Canadian Provinces</v>
+      </c>
+      <c r="D48" t="str">
+        <v>50 States listed</v>
+      </c>
+      <c r="E48" t="str">
+        <v>(full names)</v>
+      </c>
+      <c r="F48">
+        <v>0</v>
+      </c>
+      <c r="G48">
+        <v>0</v>
+      </c>
+      <c r="H48">
+        <v>0</v>
+      </c>
+      <c r="I48">
+        <v>0</v>
+      </c>
+      <c r="J48">
+        <v>0</v>
+      </c>
+      <c r="K48">
+        <v>0</v>
+      </c>
+      <c r="L48">
+        <v>0</v>
+      </c>
+      <c r="M48">
+        <v>0</v>
+      </c>
+      <c r="N48">
+        <v>0</v>
+      </c>
+      <c r="O48">
+        <v>0</v>
+      </c>
+      <c r="P48">
+        <v>0</v>
+      </c>
+      <c r="Q48">
+        <v>0</v>
+      </c>
+      <c r="R48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A49" t="str">
+        <v>Gender</v>
+      </c>
+      <c r="B49">
+        <v>0</v>
+      </c>
+      <c r="C49" t="str">
+        <v>female</v>
+      </c>
+      <c r="D49" t="str">
+        <v>male</v>
+      </c>
+      <c r="E49" t="str">
+        <v>non-binary</v>
+      </c>
+      <c r="F49" t="str">
+        <v>other (please type here)</v>
+      </c>
+      <c r="G49">
+        <v>0</v>
+      </c>
+      <c r="H49">
+        <v>0</v>
+      </c>
+      <c r="I49">
+        <v>0</v>
+      </c>
+      <c r="J49">
+        <v>0</v>
+      </c>
+      <c r="K49">
+        <v>0</v>
+      </c>
+      <c r="L49">
+        <v>0</v>
+      </c>
+      <c r="M49">
+        <v>0</v>
+      </c>
+      <c r="N49">
+        <v>0</v>
+      </c>
+      <c r="O49">
+        <v>0</v>
+      </c>
+      <c r="P49">
+        <v>0</v>
+      </c>
+      <c r="Q49">
+        <v>0</v>
+      </c>
+      <c r="R49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A50" t="str">
+        <v>EduComplete</v>
+      </c>
+      <c r="B50">
+        <v>0</v>
+      </c>
+      <c r="C50" t="str">
+        <v>elementary school</v>
+      </c>
+      <c r="D50" t="str">
+        <v>high school</v>
+      </c>
+      <c r="E50" t="str">
+        <v>undergraduate degree</v>
+      </c>
+      <c r="F50" t="str">
+        <v>graduate degree</v>
+      </c>
+      <c r="G50" t="str">
+        <v>post-graduate degree</v>
+      </c>
+      <c r="H50" t="str">
+        <v>other (please specify):</v>
+      </c>
+      <c r="I50">
+        <v>0</v>
+      </c>
+      <c r="J50">
+        <v>0</v>
+      </c>
+      <c r="K50">
+        <v>0</v>
+      </c>
+      <c r="L50">
+        <v>0</v>
+      </c>
+      <c r="M50">
+        <v>0</v>
+      </c>
+      <c r="N50">
+        <v>0</v>
+      </c>
+      <c r="O50">
+        <v>0</v>
+      </c>
+      <c r="P50">
+        <v>0</v>
+      </c>
+      <c r="Q50">
+        <v>0</v>
+      </c>
+      <c r="R50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A51" t="str">
+        <v>DegreeYear</v>
+      </c>
+      <c r="B51">
+        <v>0</v>
+      </c>
+      <c r="C51" t="str">
+        <v>I am not currently studying</v>
+      </c>
+      <c r="D51" t="str">
+        <v>First year</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Second year</v>
+      </c>
+      <c r="F51" t="str">
+        <v>Third year</v>
+      </c>
+      <c r="G51" t="str">
+        <v>Fourth year+</v>
+      </c>
+      <c r="H51" t="str">
+        <v>Other degree (please specify)</v>
+      </c>
+      <c r="I51">
+        <v>0</v>
+      </c>
+      <c r="J51" t="str">
+        <v>I am in a graduate program</v>
+      </c>
+      <c r="K51">
+        <v>0</v>
+      </c>
+      <c r="L51">
+        <v>0</v>
+      </c>
+      <c r="M51">
+        <v>0</v>
+      </c>
+      <c r="N51">
+        <v>0</v>
+      </c>
+      <c r="O51">
+        <v>0</v>
+      </c>
+      <c r="P51">
+        <v>0</v>
+      </c>
+      <c r="Q51">
+        <v>0</v>
+      </c>
+      <c r="R51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A52" t="str">
+        <v>Region</v>
+      </c>
+      <c r="B52">
+        <v>0</v>
+      </c>
+      <c r="C52" t="str">
+        <v>BC</v>
+      </c>
+      <c r="D52" t="str">
+        <v>AB</v>
+      </c>
+      <c r="E52" t="str">
+        <v>SK</v>
+      </c>
+      <c r="F52" t="str">
+        <v>MB</v>
+      </c>
+      <c r="G52" t="str">
+        <v>ON</v>
+      </c>
+      <c r="H52" t="str">
+        <v>QC</v>
+      </c>
+      <c r="I52" t="str">
+        <v>NB</v>
+      </c>
+      <c r="J52" t="str">
+        <v>PE</v>
+      </c>
+      <c r="K52" t="str">
+        <v>NS</v>
+      </c>
+      <c r="L52" t="str">
+        <v>NL</v>
+      </c>
+      <c r="M52" t="str">
+        <v>NU</v>
+      </c>
+      <c r="N52" t="str">
+        <v>NT</v>
+      </c>
+      <c r="O52" t="str">
+        <v>YT</v>
+      </c>
+      <c r="P52" t="str">
+        <v>US (for USA)</v>
+      </c>
+      <c r="Q52">
+        <v>0</v>
+      </c>
+      <c r="R52" t="str">
+        <v xml:space="preserve">all others can be lumped as OTHER </v>
+      </c>
+    </row>
+    <row r="53" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A53" t="str">
+        <v>EUI</v>
+      </c>
+      <c r="B53">
+        <v>0</v>
+      </c>
+      <c r="C53" t="str">
+        <v>0 to 18</v>
+      </c>
+      <c r="D53" t="str">
+        <v>0 is the Englsh monolingual</v>
+      </c>
+      <c r="E53" t="str">
+        <v>18 the one who never uses English in 6 contexts</v>
+      </c>
+      <c r="F53">
+        <v>0</v>
+      </c>
+      <c r="G53" t="str">
+        <v xml:space="preserve">Idea: Classes  </v>
+      </c>
+      <c r="H53" t="str">
+        <v>0, 1-3, 4-8, 9-18</v>
+      </c>
+      <c r="I53" t="str">
+        <v>or, easier, 0 and 1+ would be good</v>
+      </c>
+      <c r="J53">
+        <v>0</v>
+      </c>
+      <c r="K53">
+        <v>0</v>
+      </c>
+      <c r="L53">
+        <v>0</v>
+      </c>
+      <c r="M53">
+        <v>0</v>
+      </c>
+      <c r="N53" t="str">
+        <v>INDEXES IN YELLOW</v>
+      </c>
+      <c r="O53">
+        <v>0</v>
+      </c>
+      <c r="P53">
+        <v>0</v>
+      </c>
+      <c r="Q53">
+        <v>0</v>
+      </c>
+      <c r="R53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A54" t="str">
+        <v>DistCult</v>
+      </c>
+      <c r="B54">
+        <v>0</v>
+      </c>
+      <c r="C54" t="str">
+        <v xml:space="preserve">yes </v>
+      </c>
+      <c r="D54" t="str">
+        <v>no</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Self-identifying</v>
+      </c>
+      <c r="F54" t="str">
+        <v>(emic)</v>
+      </c>
+      <c r="G54">
+        <v>0</v>
+      </c>
+      <c r="H54">
+        <v>0</v>
+      </c>
+      <c r="I54">
+        <v>0</v>
+      </c>
+      <c r="J54">
+        <v>0</v>
+      </c>
+      <c r="K54">
+        <v>0</v>
+      </c>
+      <c r="L54">
+        <v>0</v>
+      </c>
+      <c r="M54">
+        <v>0</v>
+      </c>
+      <c r="N54">
+        <v>0</v>
+      </c>
+      <c r="O54">
+        <v>0</v>
+      </c>
+      <c r="P54">
+        <v>0</v>
+      </c>
+      <c r="Q54">
+        <v>0</v>
+      </c>
+      <c r="R54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A55" t="str">
+        <v>EOI</v>
+      </c>
+      <c r="B55">
+        <v>0</v>
+      </c>
+      <c r="C55">
+        <v>0</v>
+      </c>
+      <c r="D55" t="str">
+        <v>0 to 15 (adapted from Walker)</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Correlated with language skills</v>
+      </c>
+      <c r="F55" t="str">
+        <v xml:space="preserve">Here, no EOI means: etically not a linguistic group member </v>
+      </c>
+      <c r="G55">
+        <v>0</v>
+      </c>
+      <c r="H55">
+        <v>0</v>
+      </c>
+      <c r="I55">
+        <v>0</v>
+      </c>
+      <c r="J55">
+        <v>0</v>
+      </c>
+      <c r="K55">
+        <v>0</v>
+      </c>
+      <c r="L55">
+        <v>0</v>
+      </c>
+      <c r="M55">
+        <v>0</v>
+      </c>
+      <c r="N55">
+        <v>0</v>
+      </c>
+      <c r="O55">
+        <v>0</v>
+      </c>
+      <c r="P55">
+        <v>0</v>
+      </c>
+      <c r="Q55">
+        <v>0</v>
+      </c>
+      <c r="R55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A56" t="str">
+        <v>SocMedia</v>
+      </c>
+      <c r="B56">
+        <v>0</v>
+      </c>
+      <c r="C56" t="str">
+        <v>I don't use social media</v>
+      </c>
+      <c r="D56" t="str">
+        <v>less than 30 minutes</v>
+      </c>
+      <c r="E56" t="str">
+        <v>30 minutes to 1 hour</v>
+      </c>
+      <c r="F56" t="str">
+        <v>1-2 hours</v>
+      </c>
+      <c r="G56" t="str">
+        <v>2-4 hours</v>
+      </c>
+      <c r="H56" t="str">
+        <v>4-6 hours</v>
+      </c>
+      <c r="I56" t="str">
+        <v>6-8 hours</v>
+      </c>
+      <c r="J56" t="str">
+        <v>more than 8 hours</v>
+      </c>
+      <c r="K56">
+        <v>0</v>
+      </c>
+      <c r="L56">
+        <v>0</v>
+      </c>
+      <c r="M56">
+        <v>0</v>
+      </c>
+      <c r="N56">
+        <v>0</v>
+      </c>
+      <c r="O56">
+        <v>0</v>
+      </c>
+      <c r="P56">
+        <v>0</v>
+      </c>
+      <c r="Q56">
+        <v>0</v>
+      </c>
+      <c r="R56">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>